<commit_message>
feat: complete Excel-first learning experience
</commit_message>
<xml_diff>
--- a/examples/dirty_data.xlsx
+++ b/examples/dirty_data.xlsx
@@ -8,67 +8,91 @@
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
-    <sheet name="Auxiliar" sheetId="2" r:id="rId2"/>
+    <sheet name="Guía" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
-  <si>
-    <t>codigo</t>
-  </si>
-  <si>
-    <t>monto</t>
-  </si>
-  <si>
-    <t>porcentaje</t>
-  </si>
-  <si>
-    <t>categoria</t>
-  </si>
-  <si>
-    <t>001</t>
-  </si>
-  <si>
-    <t>002</t>
-  </si>
-  <si>
-    <t>003</t>
-  </si>
-  <si>
-    <t>1.234,50</t>
-  </si>
-  <si>
-    <t>2.100,00</t>
-  </si>
-  <si>
-    <t>999.999,00</t>
-  </si>
-  <si>
-    <t>15%</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>0.15</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+  <si>
+    <t>Registro_ID</t>
+  </si>
+  <si>
+    <t>Zona</t>
+  </si>
+  <si>
+    <t>Monto</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Constante</t>
+  </si>
+  <si>
+    <t>REG-001</t>
+  </si>
+  <si>
+    <t>REG-002</t>
+  </si>
+  <si>
+    <t>REG-003</t>
+  </si>
+  <si>
+    <t>REG-005</t>
+  </si>
+  <si>
+    <t>REG-006</t>
+  </si>
+  <si>
+    <t>Lima</t>
+  </si>
+  <si>
+    <t>lima</t>
   </si>
   <si>
     <t>Norte</t>
   </si>
   <si>
-    <t xml:space="preserve"> Sur </t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>nota</t>
-  </si>
-  <si>
-    <t>Hoja auxiliar sintética</t>
+    <t xml:space="preserve">Sur </t>
+  </si>
+  <si>
+    <t>2026-01-03</t>
+  </si>
+  <si>
+    <t>2026-01-04</t>
+  </si>
+  <si>
+    <t>2026-01-05</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
+  </si>
+  <si>
+    <t>Activo</t>
+  </si>
+  <si>
+    <t>Pausado</t>
+  </si>
+  <si>
+    <t>misma</t>
+  </si>
+  <si>
+    <t>Tema</t>
+  </si>
+  <si>
+    <t>Explicación</t>
+  </si>
+  <si>
+    <t>Uso</t>
+  </si>
+  <si>
+    <t>Workbook auxiliar para pruebas de formato y perfilado.</t>
   </si>
 </sst>
 </file>
@@ -426,10 +450,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="6" width="20.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,64 +469,122 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>120</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4">
+        <v>95.5</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
+        <v>95.5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>140</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="B6">
-        <f>SUM(1,2)</f>
-        <v>0</v>
+      <c r="C7">
+        <v>110</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -509,17 +594,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="6" width="20.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>22</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>